<commit_message>
feat: classify documents and refresh sample data
</commit_message>
<xml_diff>
--- a/sample-data/ai-cashflow-variants/01-tiem-banh-may-som/input/01_ban_hang_theo_ngay.xlsx
+++ b/sample-data/ai-cashflow-variants/01-tiem-banh-may-som/input/01_ban_hang_theo_ngay.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đọc trước" sheetId="1" r:id="R66fc2089891845e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T04" sheetId="2" r:id="Rf30b2e1ff13449c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T05" sheetId="3" r:id="R7a61c738b4ff40d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T06" sheetId="4" r:id="R89dd30af8fb2488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đọc trước" sheetId="1" r:id="R7cd722e5093e479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T04" sheetId="2" r:id="Re4f3b2230dc5400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T05" sheetId="3" r:id="R5c8fffe0632d4df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T06" sheetId="4" r:id="Rc46833c2e6aa4331"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>